<commit_message>
fix: remove linha central dos graficos e atualiza xlsx com nova cotação
- fill='tozeroy' com range explícito elimina o trace baseline desnecessário
- Título PPG sem referência a países (alterado na planilha)
- xlsx atualizado com nova cotação US$

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Posição Financeira/Posição Financeira 19-06-2026.xlsx
+++ b/data/Posição Financeira/Posição Financeira 19-06-2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailadventistas.sharepoint.com/sites/SAD-DSA-IAJA/Documentos Compartilhados/IAJA/01 - IAJA/05 - CONTABILIDADE/03 - CAIXA/09 - PLANILHAS/Posição Financeira/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailadventistas-my.sharepoint.com/personal/heber_elias_adventistas_org/Documents/pessoal/Projetos IA/VIGIA/data/Posição Financeira/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="8_{CA735DC7-0780-4D5B-902D-19CDAB62B616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5756DCE7-1A51-4C0F-AD78-A49B0118AE02}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="8_{CA735DC7-0780-4D5B-902D-19CDAB62B616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E97A35-0231-413A-8CD8-5F1F00CFC326}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8AE765BB-1B3B-C94A-80E9-FD6B0D5051C9}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8AE765BB-1B3B-C94A-80E9-FD6B0D5051C9}"/>
   </bookViews>
   <sheets>
     <sheet name="QUADRO" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="84">
   <si>
     <t>GENERAL CONFERENCE - SOUTH AMERICAN DIVISION</t>
   </si>
@@ -109,9 +109,6 @@
   </si>
   <si>
     <t>BRASIL</t>
-  </si>
-  <si>
-    <t>URUGUAI/USA</t>
   </si>
   <si>
     <t>IAJA - CONSOLIDADO</t>
@@ -775,16 +772,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>3159725139.681829</c:v>
+                  <c:v>3178670595.4822741</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3151047667.6018295</c:v>
+                  <c:v>3155419695.8634701</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3142675221.0818291</c:v>
+                  <c:v>3155791305.8667526</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3144099682.7518296</c:v>
+                  <c:v>3145557025.5057101</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>3140666122.1918287</c:v>
@@ -1261,31 +1258,31 @@
                 <c:pt idx="12">
                   <c:v>2358987689.6599998</c:v>
                 </c:pt>
-                <c:pt idx="13" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="13" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2345192562.6700001</c:v>
                 </c:pt>
-                <c:pt idx="14" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="14" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2333129232.9900002</c:v>
                 </c:pt>
-                <c:pt idx="15" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="15" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2295127222.3600001</c:v>
                 </c:pt>
-                <c:pt idx="16" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="16" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2271014228.1299996</c:v>
                 </c:pt>
-                <c:pt idx="17" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="17" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2247964340.5899997</c:v>
                 </c:pt>
-                <c:pt idx="18" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="18" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2224848776.8799996</c:v>
                 </c:pt>
-                <c:pt idx="19" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="19" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2195911180.0100002</c:v>
                 </c:pt>
-                <c:pt idx="20" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="20" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2177545979.2200003</c:v>
                 </c:pt>
-                <c:pt idx="21" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="21" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>2158908830.96</c:v>
                 </c:pt>
               </c:numCache>
@@ -1706,31 +1703,31 @@
                 <c:pt idx="12">
                   <c:v>133873608.37580818</c:v>
                 </c:pt>
-                <c:pt idx="13" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="13" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>139950615.67223063</c:v>
                 </c:pt>
-                <c:pt idx="14" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="14" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>138161808.50682876</c:v>
                 </c:pt>
-                <c:pt idx="15" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="15" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>134056646.97828791</c:v>
                 </c:pt>
-                <c:pt idx="16" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="16" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>134109695.81459738</c:v>
                 </c:pt>
-                <c:pt idx="17" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="17" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>133149254.09693986</c:v>
                 </c:pt>
-                <c:pt idx="18" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="18" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>131265644.44962728</c:v>
                 </c:pt>
-                <c:pt idx="19" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="19" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>127937272.63128272</c:v>
                 </c:pt>
-                <c:pt idx="20" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="20" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>125273440.21058296</c:v>
                 </c:pt>
-                <c:pt idx="21" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
+                <c:pt idx="21" formatCode="_-* #.##0_-;\-* #.##0_-;_-* &quot;-&quot;??_-;_-@_-">
                   <c:v>124048773.91446033</c:v>
                 </c:pt>
               </c:numCache>
@@ -4608,23 +4605,23 @@
       </c>
       <c r="L17" s="16">
         <f>Somatória!C30</f>
-        <v>61671434.357700005</v>
+        <v>63263351.124399997</v>
       </c>
       <c r="M17" s="17">
         <f>Somatória!C30/Somatória!D30-1</f>
-        <v>3.2412166306006185E-5</v>
+        <v>1.9771332188372348E-2</v>
       </c>
       <c r="N17" s="17">
         <f>Somatória!C30/Somatória!G30-1</f>
-        <v>3.7997041629855843E-4</v>
+        <v>2.6202649336652062E-2</v>
       </c>
       <c r="O17" s="17">
         <f>Somatória!C30/Somatória!N30-1</f>
-        <v>-4.1859399012321941E-2</v>
+        <v>-1.7127039477411121E-2</v>
       </c>
       <c r="P17" s="17">
         <f>Somatória!C30/Somatória!X30-1</f>
-        <v>-7.7511033275470043E-2</v>
+        <v>-5.3698944769356438E-2</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4660,23 +4657,23 @@
       </c>
       <c r="L18" s="16">
         <f>Somatória!C31</f>
-        <v>3098053705.3241291</v>
+        <v>3115407244.3578739</v>
       </c>
       <c r="M18" s="17">
         <f>Somatória!C31/Somatória!D31-1</f>
-        <v>2.808161574358925E-3</v>
+        <v>7.1198264708334236E-3</v>
       </c>
       <c r="N18" s="17">
         <f>Somatória!C31/Somatória!G31-1</f>
-        <v>6.1823582635778251E-3</v>
+        <v>1.1818420930659768E-2</v>
       </c>
       <c r="O18" s="17">
         <f>Somatória!C31/Somatória!N31-1</f>
-        <v>3.1253954119818683E-2</v>
+        <v>3.7030453641362593E-2</v>
       </c>
       <c r="P18" s="17">
         <f>Somatória!C31/Somatória!X31-1</f>
-        <v>0.10963069289275684</v>
+        <v>0.11584621443425358</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
@@ -4728,23 +4725,23 @@
       </c>
       <c r="L20" s="16">
         <f>SUM(L17:L19)</f>
-        <v>3159725139.681829</v>
+        <v>3178670595.4822741</v>
       </c>
       <c r="M20" s="19">
         <f>Somatória!C32/Somatória!D32-1</f>
-        <v>2.753837134619852E-3</v>
+        <v>7.368560083872211E-3</v>
       </c>
       <c r="N20" s="19">
         <f>Somatória!C32/Somatória!G32-1</f>
-        <v>6.0684634241539026E-3</v>
+        <v>1.210076837582541E-2</v>
       </c>
       <c r="O20" s="19">
         <f>Somatória!C32/Somatória!N32-1</f>
-        <v>2.9720320976292847E-2</v>
+        <v>3.5894440548554396E-2</v>
       </c>
       <c r="P20" s="19">
         <f>Somatória!C32/Somatória!X32-1</f>
-        <v>0.10525439933333058</v>
+        <v>0.11188141511639516</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4761,7 +4758,7 @@
         <v>15</v>
       </c>
       <c r="L21" s="24">
-        <v>5.03</v>
+        <v>5.16</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
@@ -4778,7 +4775,7 @@
         <v>16</v>
       </c>
       <c r="K23" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
@@ -4822,10 +4819,10 @@
     </row>
     <row r="37" spans="3:18" x14ac:dyDescent="0.25">
       <c r="C37" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="R37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="13:16" ht="3.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4834,12 +4831,12 @@
     </row>
     <row r="58" spans="13:16" x14ac:dyDescent="0.25">
       <c r="P58" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="59" spans="13:16" x14ac:dyDescent="0.25">
       <c r="O59" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P59" s="27">
         <f ca="1">TODAY()</f>
@@ -4971,7 +4968,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <f>Preenchimento!D10</f>
@@ -5258,7 +5255,7 @@
     </row>
     <row r="11" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>3</v>
@@ -5355,7 +5352,7 @@
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <f>Preenchimento!D37</f>
@@ -5552,7 +5549,7 @@
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15">
         <f t="shared" ref="C15:D15" si="25">((SUM(C12:C14))*1.01)*1.000235</f>
@@ -5648,7 +5645,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="7" t="str">
         <f t="shared" ref="C20" si="37">C11</f>
@@ -5742,7 +5739,7 @@
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21">
         <f>Preenchimento!D24</f>
@@ -6029,7 +6026,7 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26">
         <f t="shared" ref="C26" si="62">C6+C24</f>
@@ -6124,19 +6121,19 @@
       <c r="B30" s="28"/>
       <c r="C30" s="28">
         <f t="shared" ref="C30" si="75">C3+(C12*C35)+C21</f>
-        <v>61671434.357700005</v>
+        <v>63263351.124399997</v>
       </c>
       <c r="D30" s="28">
         <f t="shared" ref="D30:E30" si="76">D3+(D12*D35)+D21</f>
-        <v>61669435.517700002</v>
+        <v>62036800.925399989</v>
       </c>
       <c r="E30" s="28">
         <f t="shared" si="76"/>
-        <v>61693293.437700003</v>
+        <v>62795389.660799995</v>
       </c>
       <c r="F30" s="28">
         <f t="shared" ref="F30:G30" si="77">F3+(F12*F35)+F21</f>
-        <v>61770663.257700004</v>
+        <v>61893118.393599994</v>
       </c>
       <c r="G30" s="28">
         <f t="shared" si="77"/>
@@ -6215,19 +6212,19 @@
       <c r="B31" s="28"/>
       <c r="C31" s="28">
         <f t="shared" ref="C31" si="87">C4+(C13*C35)+C22</f>
-        <v>3098053705.3241291</v>
+        <v>3115407244.3578739</v>
       </c>
       <c r="D31" s="28">
         <f t="shared" ref="D31:E31" si="88">D4+(D13*D35)+D22</f>
-        <v>3089378232.0841293</v>
+        <v>3093382894.9380703</v>
       </c>
       <c r="E31" s="28">
         <f t="shared" si="88"/>
-        <v>3080981927.6441293</v>
+        <v>3092995916.2059526</v>
       </c>
       <c r="F31" s="28">
         <f t="shared" ref="F31:G31" si="89">F4+(F13*F35)+F22</f>
-        <v>3082329019.4941297</v>
+        <v>3083663907.1121101</v>
       </c>
       <c r="G31" s="28">
         <f t="shared" si="89"/>
@@ -6305,19 +6302,19 @@
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C32">
         <f t="shared" ref="C32:D32" si="100">SUM(C30:C31)</f>
-        <v>3159725139.681829</v>
+        <v>3178670595.4822741</v>
       </c>
       <c r="D32">
         <f t="shared" si="100"/>
-        <v>3151047667.6018295</v>
+        <v>3155419695.8634701</v>
       </c>
       <c r="E32">
         <f t="shared" ref="E32:F32" si="101">SUM(E30:E31)</f>
-        <v>3142675221.0818291</v>
+        <v>3155791305.8667526</v>
       </c>
       <c r="F32">
         <f t="shared" si="101"/>
-        <v>3144099682.7518296</v>
+        <v>3145557025.5057101</v>
       </c>
       <c r="G32">
         <f t="shared" ref="G32:O32" si="102">SUM(G30:G31)</f>
@@ -6394,22 +6391,22 @@
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" t="s">
         <v>26</v>
       </c>
-      <c r="B35" t="s">
-        <v>27</v>
-      </c>
       <c r="C35">
-        <v>5.03</v>
+        <v>5.16</v>
       </c>
       <c r="D35">
-        <v>5.03</v>
+        <v>5.0599999999999996</v>
       </c>
       <c r="E35">
-        <v>5.03</v>
+        <v>5.12</v>
       </c>
       <c r="F35">
-        <v>5.03</v>
+        <v>5.04</v>
       </c>
       <c r="G35">
         <v>5.03</v>
@@ -6506,93 +6503,93 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="35" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" t="s">
+        <v>76</v>
+      </c>
+      <c r="M1" t="s">
+        <v>77</v>
+      </c>
+      <c r="N1" t="s">
+        <v>78</v>
+      </c>
+      <c r="O1" t="s">
+        <v>79</v>
+      </c>
+      <c r="P1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q1" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="R1" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="S1" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="T1" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="V1" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="W1" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="X1" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y1" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="35" t="s">
-        <v>84</v>
-      </c>
-      <c r="E1" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="35" t="s">
-        <v>82</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="I1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K1" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" t="s">
-        <v>77</v>
-      </c>
-      <c r="M1" t="s">
-        <v>78</v>
-      </c>
-      <c r="N1" t="s">
-        <v>79</v>
-      </c>
-      <c r="O1" t="s">
-        <v>80</v>
-      </c>
-      <c r="P1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q1" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="R1" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="S1" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="T1" s="31" t="s">
-        <v>34</v>
-      </c>
-      <c r="U1" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="V1" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="W1" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="X1" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y1" s="31" t="s">
+      <c r="Z1" s="31" t="s">
         <v>30</v>
-      </c>
-      <c r="Z1" s="31" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2">
         <v>1181</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2">
         <v>20000</v>
@@ -6666,13 +6663,13 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>2271</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" s="29">
         <v>5000</v>
@@ -6746,13 +6743,13 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>2271</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="29">
         <v>5000</v>
@@ -6826,13 +6823,13 @@
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5">
         <v>2271</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" s="29">
         <v>5000</v>
@@ -6906,13 +6903,13 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6">
         <v>2271</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="29">
         <v>5000</v>
@@ -6986,13 +6983,13 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>3100</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7">
         <v>5000</v>
@@ -7066,13 +7063,13 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8">
         <v>3100</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D8">
         <v>1000</v>
@@ -7147,13 +7144,13 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9">
         <v>3100</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D9">
         <v>500</v>
@@ -7336,10 +7333,10 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="s">
         <v>46</v>
-      </c>
-      <c r="B12" t="s">
-        <v>47</v>
       </c>
       <c r="Q12" s="26"/>
       <c r="R12" s="26"/>
@@ -7354,10 +7351,10 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
         <v>48</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
       </c>
       <c r="C13" s="29"/>
       <c r="D13" s="29">
@@ -7433,10 +7430,10 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" t="s">
         <v>50</v>
-      </c>
-      <c r="B14" t="s">
-        <v>51</v>
       </c>
       <c r="D14" s="29">
         <v>604559397.63999999</v>
@@ -7512,10 +7509,10 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
         <v>52</v>
-      </c>
-      <c r="B15" t="s">
-        <v>53</v>
       </c>
       <c r="D15" s="29">
         <v>287176148.88999999</v>
@@ -7591,10 +7588,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
         <v>54</v>
-      </c>
-      <c r="B16" t="s">
-        <v>55</v>
       </c>
       <c r="D16" s="29">
         <f>17312408.24-42460.15</f>
@@ -7672,7 +7669,7 @@
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B17" s="32">
         <v>1020308010100</v>
@@ -7859,7 +7856,7 @@
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q20" s="26"/>
       <c r="R20" s="26"/>
@@ -7874,13 +7871,13 @@
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
         <v>28</v>
-      </c>
-      <c r="C21" t="s">
-        <v>29</v>
       </c>
       <c r="Q21" s="26"/>
       <c r="R21" s="26"/>
@@ -7895,13 +7892,13 @@
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22">
         <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="29">
         <v>30000</v>
@@ -7975,13 +7972,13 @@
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23">
         <v>3416</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -8050,7 +8047,7 @@
         <v>37.01</v>
       </c>
       <c r="Z23" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.25">
@@ -8164,10 +8161,10 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" t="s">
         <v>46</v>
-      </c>
-      <c r="B26" t="s">
-        <v>47</v>
       </c>
       <c r="Q26" s="26"/>
       <c r="R26" s="26"/>
@@ -8182,10 +8179,10 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D27" s="29">
         <v>38962184.119999997</v>
@@ -8272,10 +8269,10 @@
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D28" s="29">
         <v>80818509.930000007</v>
@@ -8352,10 +8349,10 @@
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
         <v>62</v>
-      </c>
-      <c r="B29" t="s">
-        <v>63</v>
       </c>
       <c r="C29">
         <v>12823624</v>
@@ -8434,7 +8431,7 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B30">
         <v>1219001</v>
@@ -8515,10 +8512,10 @@
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" t="s">
         <v>65</v>
-      </c>
-      <c r="B31" t="s">
-        <v>66</v>
       </c>
       <c r="D31" s="30">
         <f>7746718.47+1200000</f>
@@ -8614,10 +8611,10 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" t="s">
         <v>67</v>
-      </c>
-      <c r="B32" t="s">
-        <v>68</v>
       </c>
       <c r="D32">
         <f>32941102.36+129119762.71</f>
@@ -8837,104 +8834,104 @@
     </row>
     <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" t="s">
         <v>28</v>
       </c>
-      <c r="C36" t="s">
-        <v>29</v>
-      </c>
       <c r="D36" t="str">
-        <f>D1</f>
+        <f t="shared" ref="D36:I36" si="54">D1</f>
         <v>03/Junho</v>
       </c>
       <c r="E36" t="str">
-        <f>E1</f>
+        <f t="shared" si="54"/>
         <v>02/Junho</v>
       </c>
       <c r="F36" t="str">
-        <f>F1</f>
+        <f t="shared" si="54"/>
         <v>01/Junho</v>
       </c>
       <c r="G36" t="str">
-        <f>G1</f>
+        <f t="shared" si="54"/>
         <v>04/Maio</v>
       </c>
       <c r="H36" t="str">
-        <f>H1</f>
+        <f t="shared" si="54"/>
         <v>03/Maio</v>
       </c>
       <c r="I36" t="str">
-        <f>I1</f>
+        <f t="shared" si="54"/>
         <v>02/Maio</v>
       </c>
       <c r="J36" t="str">
-        <f t="shared" ref="J36:P36" si="54">J1</f>
+        <f t="shared" ref="J36:P36" si="55">J1</f>
         <v>01/Maio</v>
       </c>
       <c r="K36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>05/Abril</v>
       </c>
       <c r="L36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>04/Abril</v>
       </c>
       <c r="M36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>03/Abril</v>
       </c>
       <c r="N36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02/Abril</v>
       </c>
       <c r="O36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>01/Abril</v>
       </c>
       <c r="P36" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>04/Março</v>
       </c>
       <c r="Q36" s="26" t="str">
-        <f t="shared" ref="Q36" si="55">Q1</f>
+        <f t="shared" ref="Q36" si="56">Q1</f>
         <v>04/Fevereiro</v>
       </c>
       <c r="R36" s="26" t="str">
-        <f t="shared" ref="R36" si="56">R1</f>
+        <f t="shared" ref="R36" si="57">R1</f>
         <v>04/Janeiro</v>
       </c>
       <c r="S36" s="26" t="str">
-        <f t="shared" ref="S36" si="57">S1</f>
+        <f t="shared" ref="S36" si="58">S1</f>
         <v>05/Dezembro</v>
       </c>
       <c r="T36" s="26" t="str">
-        <f t="shared" ref="T36" si="58">T1</f>
+        <f t="shared" ref="T36" si="59">T1</f>
         <v>04/Novembro</v>
       </c>
       <c r="U36" s="26" t="str">
-        <f t="shared" ref="U36" si="59">U1</f>
+        <f t="shared" ref="U36" si="60">U1</f>
         <v>04/Outubro</v>
       </c>
       <c r="V36" s="26" t="str">
-        <f t="shared" ref="V36" si="60">V1</f>
+        <f t="shared" ref="V36" si="61">V1</f>
         <v>04/Setembro</v>
       </c>
       <c r="W36" s="26" t="str">
-        <f t="shared" ref="W36" si="61">W1</f>
+        <f t="shared" ref="W36" si="62">W1</f>
         <v>04/Agosto</v>
       </c>
       <c r="X36" s="26" t="str">
-        <f t="shared" ref="X36" si="62">X1</f>
+        <f t="shared" ref="X36" si="63">X1</f>
         <v>04/Julho</v>
       </c>
       <c r="Y36" s="26" t="str">
-        <f t="shared" ref="Y36" si="63">Y1</f>
+        <f t="shared" ref="Y36" si="64">Y1</f>
         <v>04/Junho</v>
       </c>
       <c r="Z36" s="26" t="str">
-        <f t="shared" ref="Z36" si="64">Z1</f>
+        <f t="shared" ref="Z36" si="65">Z1</f>
         <v>04/Maio</v>
       </c>
     </row>
@@ -9012,10 +9009,10 @@
     <row r="38" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="26" t="s">
         <v>46</v>
-      </c>
-      <c r="B39" s="26" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:26" s="26" customFormat="1" x14ac:dyDescent="0.25">
@@ -9105,6 +9102,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="546f6921-c430-45e7-8b30-d6d9b86d8f0f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="364167a4-bc77-49ec-93f2-879d4481bae7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F9EA5E59716CA04482326D7D6394CBC5" ma:contentTypeVersion="18" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="f5d419073af479a9667be57ebdabf5b3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="546f6921-c430-45e7-8b30-d6d9b86d8f0f" xmlns:ns3="364167a4-bc77-49ec-93f2-879d4481bae7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb422b1d84a34ba11f054fd3b754dea3" ns2:_="" ns3:_="">
     <xsd:import namespace="546f6921-c430-45e7-8b30-d6d9b86d8f0f"/>
@@ -9359,17 +9367,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="546f6921-c430-45e7-8b30-d6d9b86d8f0f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="364167a4-bc77-49ec-93f2-879d4481bae7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5656E7FC-8739-4AA4-8E2F-8E1DDD7713FD}">
   <ds:schemaRefs>
@@ -9379,6 +9376,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95E1F151-0F5C-495E-9947-EE9B49CBAA94}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="546f6921-c430-45e7-8b30-d6d9b86d8f0f"/>
+    <ds:schemaRef ds:uri="364167a4-bc77-49ec-93f2-879d4481bae7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E13DAF4-75CF-4CAD-98E0-C37001267BD0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9395,15 +9403,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95E1F151-0F5C-495E-9947-EE9B49CBAA94}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="546f6921-c430-45e7-8b30-d6d9b86d8f0f"/>
-    <ds:schemaRef ds:uri="364167a4-bc77-49ec-93f2-879d4481bae7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>